<commit_message>
feat(cp1): mark case file sections read in 0_Đầu vào
- Mark B5:B10 as "Có" with verified notes in E5:E10 on 0_Đầu vào
- Verify B12 formula equals 6/6 and column O shows "Có" for all 7 tasks
- Initialize personal QA & integration report for Pham Thanh Dat (2A202602721)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5aesieunhan_CS13.xlsx
+++ b/5aesieunhan_CS13.xlsx
@@ -774,7 +774,11 @@
           <t>Số liệu kinh tế của đề (9 dòng)</t>
         </is>
       </c>
-      <c r="B5" s="40" t="n"/>
+      <c r="B5" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C5" s="39" t="inlineStr">
         <is>
           <t>Đã điền sẵn ở trang 2, dòng 12–20: chi phí mỗi việc, biên lợi nhuận, điều kiện dừng</t>
@@ -785,7 +789,11 @@
           <t>Đọc để hiểu; không cần chép</t>
         </is>
       </c>
-      <c r="E5" s="40" t="n"/>
+      <c r="E5" s="40" t="inlineStr">
+        <is>
+          <t>Đã đối chiếu 9 dòng số liệu với trang 2 B12:B20; khớp hồ sơ</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="33.75" customHeight="1" s="33">
       <c r="A6" s="39" t="inlineStr">
@@ -793,7 +801,11 @@
           <t>Bối cảnh, sản phẩm, "1 việc" là gì</t>
         </is>
       </c>
-      <c r="B6" s="40" t="n"/>
+      <c r="B6" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
           <t>Giả thuyết và chỉ số ở trang 1</t>
@@ -804,7 +816,11 @@
           <t>Viết giả thuyết theo đúng "1 việc" của đề</t>
         </is>
       </c>
-      <c r="E6" s="40" t="n"/>
+      <c r="E6" s="40" t="inlineStr">
+        <is>
+          <t>1 việc = 1 bài viết được chấm điểm và có nhận xét; ~1.500 bài/tuần</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="33.75" customHeight="1" s="33">
       <c r="A7" s="39" t="inlineStr">
@@ -812,7 +828,11 @@
           <t>6 việc gợi ý</t>
         </is>
       </c>
-      <c r="B7" s="40" t="n"/>
+      <c r="B7" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C7" s="39" t="inlineStr">
         <is>
           <t>Trang 1, cột B–C; nhóm được thêm việc của mình</t>
@@ -823,7 +843,11 @@
           <t>Giữ, bỏ hay đổi thứ tự đều phải ghi lý do ở cột Q</t>
         </is>
       </c>
-      <c r="E7" s="40" t="n"/>
+      <c r="E7" s="40" t="inlineStr">
+        <is>
+          <t>Giữ 6 việc gợi ý, thêm việc 7 (báo cáo độ lệch cho đối tác)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="33.75" customHeight="1" s="33">
       <c r="A8" s="39" t="inlineStr">
@@ -831,7 +855,11 @@
           <t>Kết quả đánh giá đã có (bộ đề, cổng phát hành)</t>
         </is>
       </c>
-      <c r="B8" s="40" t="n"/>
+      <c r="B8" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
           <t>Cổng đánh giá ở trang 2; việc cần làm trước ở trang 3</t>
@@ -842,7 +870,11 @@
           <t>Đề 2, 3: kết luận chưa phải "Phát hành" → có việc phải làm trước</t>
         </is>
       </c>
-      <c r="E8" s="40" t="n"/>
+      <c r="E8" s="40" t="inlineStr">
+        <is>
+          <t>Phát hành có giới hạn; tầng Khó tụt 1 → sửa và chạy lại trước khi mở rộng</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="33.75" customHeight="1" s="33">
       <c r="A9" s="39" t="inlineStr">
@@ -850,7 +882,11 @@
           <t>Chuyên gia và số giờ của họ</t>
         </is>
       </c>
-      <c r="B9" s="40" t="n"/>
+      <c r="B9" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C9" s="39" t="inlineStr">
         <is>
           <t>Dòng "Điều kiện cần" ở trang 3; ô "Cần gì" ở trang 5</t>
@@ -861,7 +897,11 @@
           <t>Dẫn đúng số giờ trong hồ sơ</t>
         </is>
       </c>
-      <c r="E9" s="40" t="n"/>
+      <c r="E9" s="40" t="inlineStr">
+        <is>
+          <t>Cô Lan + thầy Khoa, 2 giờ/tuần mỗi người; 1 vòng 40 bài = 14,2 giờ</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="33.75" customHeight="1" s="33">
       <c r="A10" s="39" t="inlineStr">
@@ -869,7 +909,11 @@
           <t>Gợi ý về người duyệt và mức tự động</t>
         </is>
       </c>
-      <c r="B10" s="40" t="n"/>
+      <c r="B10" s="40" t="inlineStr">
+        <is>
+          <t>Có</t>
+        </is>
+      </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
           <t>Trang 2, cột H và I</t>
@@ -880,7 +924,11 @@
           <t>Đề 3: bác sĩ của bệnh viện không tính vào chi phí</t>
         </is>
       </c>
-      <c r="E10" s="40" t="n"/>
+      <c r="E10" s="40" t="inlineStr">
+        <is>
+          <t>Người duyệt = giáo viên công ty trả tiền; hai giáo viên giỏi khớp ~70% trong 0,5 điểm</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="33">
       <c r="A12" s="41" t="inlineStr">

</xml_diff>

<commit_message>
fix(cp3): align double-grading timeline with expert hours
- Shift double-grading to company-paid reviewer teachers at ~30 essays/week
- Update 2_Mức tự động!F7 and 3_Bảng lộ trình!C10 to reflect 4-week timeline
- Verify unit economics, break-even review threshold (17.75%), and 3/n rule
- Document resolution of expert workload contradiction in QA report

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/5aesieunhan_CS13.xlsx
+++ b/5aesieunhan_CS13.xlsx
@@ -1925,7 +1925,7 @@
       </c>
       <c r="F7" s="40" t="inlineStr">
         <is>
-          <t>Đã có mẫu chấm đôi đủ 100 bài (khoảng 5 tuần); báo cáo độ lệch gửi được cho đối tác; nhật ký bài chuyển giáo viên</t>
+          <t>Đã có mẫu chấm đôi đủ 100 bài thật: giáo viên duyệt của công ty chấm đôi (3 phút/bài, đã tính trong chi phí), chuyên gia chỉ rà bài lệch và xác nhận cổng; 2% × 1.500 bài/tuần ≈ 30 bài/tuần → khoảng 4 tuần; báo cáo độ lệch gửi được cho đối tác; nhật ký bài chuyển giáo viên</t>
         </is>
       </c>
       <c r="G7" s="40" t="inlineStr">
@@ -2363,7 +2363,7 @@
       </c>
       <c r="C10" s="40" t="inlineStr">
         <is>
-          <t>Cần ≥100 bài chấm đôi (khoảng 5 tuần); báo cáo độ lệch cho đối tác; dữ liệu điểm học sinh bắt đầu đủ sau khoảng 3 tháng.</t>
+          <t>Cần ≥100 bài chấm đôi (giáo viên duyệt của công ty chấm đôi ~30 bài/tuần, khoảng 4 tuần; chuyên gia chỉ xác nhận); báo cáo độ lệch cho đối tác; dữ liệu điểm học sinh bắt đầu đủ sau khoảng 3 tháng.</t>
         </is>
       </c>
       <c r="D10" s="40" t="inlineStr">

</xml_diff>